<commit_message>
Corrida | SFE-ART | 2026-06-19 10:49:04.292113
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ART_out.xlsx
+++ b/indicadores/SFE-ART_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">17/06/2026</t>
+    <t xml:space="preserve">19/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">focampo</t>
+    <t xml:space="preserve">fleiva</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2056,9 +2056,7 @@
       <c r="J7" s="1"/>
     </row>
     <row r="8">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
+      <c r="A8"/>
       <c r="B8"/>
       <c r="C8"/>
       <c r="D8"/>
@@ -2070,14 +2068,10 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
+      <c r="A9"/>
       <c r="B9"/>
       <c r="C9"/>
-      <c r="D9" t="n">
-        <v>0.590994003702063</v>
-      </c>
+      <c r="D9"/>
       <c r="E9"/>
       <c r="F9"/>
       <c r="G9"/>
@@ -2087,13 +2081,11 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
+      <c r="D10"/>
       <c r="E10"/>
       <c r="F10"/>
       <c r="G10"/>
@@ -2102,10 +2094,14 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11">
-      <c r="A11"/>
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
       <c r="B11"/>
       <c r="C11"/>
-      <c r="D11"/>
+      <c r="D11" t="n">
+        <v>0.589807410943029</v>
+      </c>
       <c r="E11"/>
       <c r="F11"/>
       <c r="G11"/>
@@ -2115,11 +2111,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
-      <c r="D12"/>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
       <c r="E12"/>
       <c r="F12"/>
       <c r="G12"/>
@@ -2128,14 +2126,10 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13">
-      <c r="A13" t="s">
-        <v>25</v>
-      </c>
+      <c r="A13"/>
       <c r="B13"/>
       <c r="C13"/>
-      <c r="D13" t="n">
-        <v>0.272247677082019</v>
-      </c>
+      <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
       <c r="G13"/>
@@ -2144,7 +2138,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14">
-      <c r="A14"/>
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
       <c r="B14"/>
       <c r="C14"/>
       <c r="D14"/>
@@ -2157,11 +2153,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
-      <c r="D15"/>
+      <c r="D15" t="n">
+        <v>0.264830815862165</v>
+      </c>
       <c r="E15"/>
       <c r="F15"/>
       <c r="G15"/>
@@ -2170,9 +2168,7 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16">
-      <c r="A16" t="s">
-        <v>27</v>
-      </c>
+      <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
@@ -2185,7 +2181,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2199,13 +2195,11 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
-      <c r="D18" t="n">
-        <v>0.00723795236972917</v>
-      </c>
+      <c r="D18"/>
       <c r="E18"/>
       <c r="F18"/>
       <c r="G18"/>
@@ -2215,7 +2209,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2234,7 +2228,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000000421624184230302</v>
+        <v>0.00484744534405667</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2244,7 +2238,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
       <c r="B21"/>
       <c r="C21"/>
       <c r="D21"/>
@@ -2256,10 +2252,14 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22">
-      <c r="A22"/>
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
       <c r="B22"/>
       <c r="C22"/>
-      <c r="D22"/>
+      <c r="D22" t="n">
+        <v>0.000000225864352802819</v>
+      </c>
       <c r="E22"/>
       <c r="F22"/>
       <c r="G22"/>
@@ -25089,7 +25089,7 @@
         <v>489</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.223308734291404</v>
+        <v>0.226852785450844</v>
       </c>
     </row>
     <row r="6">
@@ -25097,7 +25097,7 @@
         <v>490</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.241776398275773</v>
+        <v>0.247332851205899</v>
       </c>
     </row>
     <row r="7">
@@ -25105,7 +25105,7 @@
         <v>491</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.297893072059379</v>
+        <v>0.300376952812981</v>
       </c>
     </row>
     <row r="8">
@@ -25113,7 +25113,7 @@
         <v>492</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.307591315640753</v>
+        <v>0.307265352689927</v>
       </c>
     </row>
     <row r="9">
@@ -25121,7 +25121,7 @@
         <v>493</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.352294949050147</v>
+        <v>0.347415733534821</v>
       </c>
     </row>
     <row r="10">
@@ -25129,7 +25129,7 @@
         <v>494</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.406074325806608</v>
+        <v>0.401219350027059</v>
       </c>
     </row>
     <row r="11">
@@ -25137,7 +25137,7 @@
         <v>495</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.458485005346421</v>
+        <v>0.456026694779626</v>
       </c>
     </row>
     <row r="12">
@@ -25145,7 +25145,7 @@
         <v>496</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.452307350673784</v>
+        <v>0.4505445426894</v>
       </c>
     </row>
     <row r="13">
@@ -25153,7 +25153,7 @@
         <v>497</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.512518007802548</v>
+        <v>0.508813012519717</v>
       </c>
     </row>
     <row r="14">
@@ -25161,7 +25161,7 @@
         <v>498</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.521773587949811</v>
+        <v>0.514617154652043</v>
       </c>
     </row>
     <row r="15">
@@ -25169,7 +25169,7 @@
         <v>499</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.554113339600588</v>
+        <v>0.549932750188305</v>
       </c>
     </row>
     <row r="16">
@@ -25177,7 +25177,7 @@
         <v>500</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.590994003702063</v>
+        <v>0.589807410943029</v>
       </c>
     </row>
     <row r="17">
@@ -25185,7 +25185,7 @@
         <v>501</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.569532384405834</v>
+        <v>0.571888731315396</v>
       </c>
     </row>
     <row r="18">
@@ -25193,7 +25193,7 @@
         <v>502</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.527247682474034</v>
+        <v>0.529280074472387</v>
       </c>
     </row>
     <row r="19">
@@ -25201,7 +25201,7 @@
         <v>503</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.503763076840418</v>
+        <v>0.506651755269441</v>
       </c>
     </row>
     <row r="20">
@@ -25209,7 +25209,7 @@
         <v>504</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.447700104597766</v>
+        <v>0.452727058747685</v>
       </c>
     </row>
     <row r="21">
@@ -25217,7 +25217,7 @@
         <v>505</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.356322492220596</v>
+        <v>0.361446525284043</v>
       </c>
     </row>
     <row r="22">
@@ -25225,7 +25225,7 @@
         <v>506</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.293403702981011</v>
+        <v>0.293696974547252</v>
       </c>
     </row>
     <row r="23">
@@ -25233,7 +25233,7 @@
         <v>507</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.238495418005237</v>
+        <v>0.234352644194753</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-ART | 2026-08-11 10:39:31.8129
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ART_out.xlsx
+++ b/indicadores/SFE-ART_out.xlsx
@@ -24925,237 +24925,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA4B4641-1C37-48D4-99A7-E8C859785D87}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7ECE13D5-CDFE-463C-AE87-FC9C2190DE70}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0447111D-80B1-479F-AD5C-0CC8D5CF9198}"/>
 </file>
</xml_diff>